<commit_message>
data: re-parsed MI355X trace with multi-EP fix
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/mi355x_dsr_mxfp4/mi355x_dsr_mxfp4_mtp0_ep4_tp4_rocm711_profiling/decode_breakdown.xlsx
+++ b/results/mi355x_dsr_mxfp4/mi355x_dsr_mxfp4_mtp0_ep4_tp4_rocm711_profiling/decode_breakdown.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -471,22 +471,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>56.639</v>
+        <v>15.759</v>
       </c>
       <c r="D2" t="n">
-        <v>65.59999999999999</v>
+        <v>4</v>
       </c>
       <c r="E2" t="n">
-        <v>62.358</v>
+        <v>21.238</v>
       </c>
       <c r="F2" t="n">
-        <v>72.3</v>
+        <v>5.4</v>
       </c>
       <c r="G2" t="n">
-        <v>33.41473170731707</v>
+        <v>29.01315517241379</v>
       </c>
       <c r="H2" t="n">
-        <v>39.22939024390244</v>
+        <v>34.52398275862069</v>
       </c>
     </row>
     <row r="3">
@@ -496,19 +496,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5.719</v>
+        <v>5.479</v>
       </c>
       <c r="D3" t="n">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="G3" t="n">
-        <v>5.814658536585366</v>
+        <v>5.510827586206896</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>model.layers.20.self_attn.fused_qkv_a_proj</t>
+          <t>gemm_a16w16</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -517,82 +517,552 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>18.279</v>
+        <v>15.92</v>
       </c>
       <c r="D4" t="n">
-        <v>21.2</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
-        <v>18.279</v>
+        <v>15.92</v>
       </c>
       <c r="F4" t="n">
-        <v>21.2</v>
+        <v>4</v>
       </c>
       <c r="G4" t="n">
-        <v>16.22151219512195</v>
+        <v>16.07017241379311</v>
       </c>
       <c r="H4" t="n">
-        <v>16.22151219512195</v>
+        <v>16.07017241379311</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>hipLaunchKernel</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>void aiter::add_rmsnorm_quant_kernel&lt;std::bfloat16_t, std::bfloat16_t, 256, 8, false, false, true, 1&gt;(std::bfloat16_t*, std::bfloat16_t*, float*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, double, int, int, int, int, int, int, int, bool)</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>5.479</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>10.998</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5.479017241379311</v>
+      </c>
+      <c r="H5" t="n">
+        <v>10.90012068965517</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>void aiter::add_rmsnorm_quant_kernel&lt;std::bfloat16_t, std::bfloat16_t, 64, 8, false, false, true, 1&gt;(std::bfloat16_t*, std::bfloat16_t*, float*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, double, int, int, int, int, int, int, int, bool)</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5.421103448275861</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>q_proj_and_k_up_proj</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Cijk_Alik_Bljk_BBS_BH_Bias_HA_S_SAV_UserArgs_MT64x32x128_MI16x16x1_SN_LDSB1_AFC1_AFEM1_AFEM1_ASEM1_CLR1_CADS0_DTLA0_DTLB0_DTVA0_DTVB0_EPS0_FDSI0_GRPM1_GRVWA8_GRVWB8_GSU0_GSUAMB_GLS0_ISA950_IU1_K1_LBSPPA512_LBSPPB256_LBSPPM0_LPA16_LPB16_LPM0_LRVW8_LWPMn1_MIAV0_MIWT2_1_MO40_NTn1_NTA0_NTB0_NTC0_NTD0_NTM0_NEPBS0_NLCA1_NLCB1_ONLL1_PGR2_PLR1_PKA1_SIA3_SS1_SPO0_SRVW0_SSO0_SVW2_SK3_SKXCCM8_TLDS1_ULSGRO0_USL1_UIOFGRO0_USFGRO0_VSn1_VWA2_VWB1_WSGRA0_WSGRB0_WS64_WG32_8_1</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>10.879</v>
+      </c>
+      <c r="D7" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="E7" t="n">
+        <v>16.398</v>
+      </c>
+      <c r="F7" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>11.7866724137931</v>
+      </c>
+      <c r="H7" t="n">
+        <v>17.25743103448276</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>_batched_gemm_a8w8_a_per_token_group_prequant_w_per_batched_tensor_quant_kernel_HAS_BIAS_0_BLOCK_SIZE_M_32_BLOCK_SIZE_N_128_BLOCK_SIZE_K_128_GROUP_SIZE_M_1_EVEN_K_1_EVEN_MN_1_cache_modifier_CG</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>5.470758620689654</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>rope_and_kv_cache</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>void aiter::fuse_qk_rope_concat_and_cache_mla_per_head_kernel&lt;std::bfloat16_t, _BitInt(8), _BitInt(8), (vllm::Fp8KVCacheDataType)1, (vllm::Fp8KVCacheDataType)1, 8&gt;(std::bfloat16_t const*, std::bfloat16_t const*, std::bfloat16_t const*, std::bfloat16_t const*, _BitInt(8)*, _BitInt(8)*, long const*, long const*, std::bfloat16_t const*, std::bfloat16_t const*, int, int, int, int, int, int, int, int, int, int, int, int, int, int, float const*, float const*, bool, bool)</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5.359</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5.359</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5.276948275862069</v>
+      </c>
+      <c r="H9" t="n">
+        <v>5.276948275862069</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>mla_decode</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>aiter::mla_a8w8_qh16_qseqlen1_gqaratio16_ps</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>25.319</v>
+      </c>
+      <c r="D10" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>31.918</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>25.52596551724138</v>
+      </c>
+      <c r="H10" t="n">
+        <v>32.72358620689656</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>void kn_mla_reduce_v1_ps&lt;MlaReduceKernelV1Traits&lt;512, 16, 1&gt;, float, std::bfloat16_t&gt;(MlaReduceKernelV1Params)</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>6.599</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="G11" t="n">
+        <v>7.197620689655173</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>v_up_proj_and_o_proj</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>_batched_gemm_a8w8_a_per_token_group_prequant_w_per_batched_tensor_quant_kernel_HAS_BIAS_0_BLOCK_SIZE_M_32_BLOCK_SIZE_N_64_BLOCK_SIZE_K_128_GROUP_SIZE_M_1_EVEN_K_1_EVEN_MN_1_cache_modifier_CG</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5.439</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>25.718</v>
+      </c>
+      <c r="F12" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>6.559741379310346</v>
+      </c>
+      <c r="H12" t="n">
+        <v>27.92168965517241</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Cijk_Alik_Bljk_BBS_BH_Bias_HA_S_SAV_UserArgs_MT64x64x128_MI16x16x1_SN_LDSB1_AFC1_AFEM1_AFEM1_ASEM1_CLR1_CADS0_DTLA0_DTLB0_DTVA0_DTVB0_EPS0_FDSI0_GRPM1_GRVWA8_GRVWB8_GSU0_GSUAMB_GLS0_ISA950_IU1_K1_LBSPPA512_LBSPPB512_LBSPPM0_LPA16_LPB16_LPM0_LRVW8_LWPMn1_MIAV0_MIWT2_2_MO40_NTn1_NTA0_NTB0_NTC0_NTD0_NTM0_NEPBS0_NLCA1_NLCB1_ONLL1_PGR2_PLR1_PKA1_SIA3_SS1_SPO0_SRVW0_SSO0_SVW2_SK3_SKXCCM8_TLDS1_ULSGRO0_USL1_UIOFGRO0_USFGRO0_VSn1_VWA2_VWB2_WSGRA0_WSGRB0_WS64_WG32_8_1</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>20.279</v>
+      </c>
+      <c r="D13" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G13" t="n">
+        <v>21.36194827586207</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>triton_poi_fused_as_strided_clone_copy__0</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>triton_poi_fused_as_strided_clone_copy__0</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6.479</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="E14" t="n">
+        <v>6.479</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5.486</v>
+      </c>
+      <c r="H14" t="n">
+        <v>5.486</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>post_attn_layernorm</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>void aiter::add_rmsnorm_quant_kernel&lt;std::bfloat16_t, std::bfloat16_t, 256, 8, false, false, true, 1&gt;(std::bfloat16_t*, std::bfloat16_t*, float*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, double, int, int, int, int, int, int, int, bool)</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>5.639</v>
-      </c>
-      <c r="D5" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="E5" t="n">
-        <v>5.639</v>
-      </c>
-      <c r="F5" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="G5" t="n">
-        <v>5.762926829268292</v>
-      </c>
-      <c r="H5" t="n">
-        <v>5.762926829268292</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>void aiter::reduce_scatter_cross_device_store&lt;std::bfloat16_t, 4&gt;(aiter::RankData*, aiter::RankSignals, aiter::Signal*, int, int)</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>19.959</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" t="n">
+        <v>25.278</v>
+      </c>
+      <c r="F15" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="G15" t="n">
+        <v>20.01237931034483</v>
+      </c>
+      <c r="H15" t="n">
+        <v>25.68727586206897</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>void aiter::local_device_load_rmsnorm&lt;std::bfloat16_t, 512, 2&gt;(aiter::RankSignals, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, float, int, int, int)</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>5.319</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G16" t="n">
+        <v>5.674896551724138</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>triton_poi_fused_as_strided_clone_1</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>triton_poi_fused_as_strided_clone_1</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="D17" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E17" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G17" t="n">
+        <v>5.474241379310344</v>
+      </c>
+      <c r="H17" t="n">
+        <v>5.474241379310344</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>gemm_a16w16</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>aiter::bf16gemm_fp32bf16_tn_64x64_splitk_clean</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="D18" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="E18" t="n">
+        <v>9.24</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="G18" t="n">
+        <v>9.248000000000001</v>
+      </c>
+      <c r="H18" t="n">
+        <v>9.248000000000001</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>rocm_aiter_biased_grouped_topk_impl</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>void aiter::grouped_topk_opt_sort_kernel&lt;c10::BFloat16, float __vector(4), 8, true, true, false&gt;(c10::BFloat16*, c10::BFloat16 const*, float*, int*, unsigned long, int, int, int, int, float)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>5.319</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E19" t="n">
+        <v>221.394</v>
+      </c>
+      <c r="F19" t="n">
+        <v>56</v>
+      </c>
+      <c r="G19" t="n">
+        <v>5.37351724137931</v>
+      </c>
+      <c r="H19" t="n">
+        <v>208.8833620689655</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>void ck_tile::kentry&lt;2, ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;, ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;::Kargs&gt;(ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;::Kargs)</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>6.519</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G20" t="n">
+        <v>5.394896551724138</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>void ck_tile::kentry&lt;2, ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;, ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;::Kargs&gt;(ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;::Kargs)</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>6.519</v>
+      </c>
+      <c r="D21" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="G21" t="n">
+        <v>5.395620689655173</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>_fused_dynamic_mxfp4_quant_moe_sort_kernel</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>9.519</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G22" t="n">
+        <v>9.472137931034483</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>void ck::kernel_moe_mxgemm_2lds&lt;ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 256, 64, 128, 128, 16, 16, 16, 16, 4, 2, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 32, 1, 8&gt;, ck::Sequence&lt;8, 1, 8&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)2, 1, false, true, false, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;, true, (ck::InMemoryDataOperationEnum)0, 2, (ck::TailNumber)1&gt;(ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 256, 64, 128, 128, 16, 16, 16, 16, 4, 2, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 32, 1, 8&gt;, ck::Sequence&lt;8, 1, 8&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)2, 1, false, true, false, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;::Argument)</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>123.76</v>
+      </c>
+      <c r="D23" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="G23" t="n">
+        <v>119.4599137931035</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>_fused_dynamic_mxfp4_quant_moe_sort_kernel</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>6.079</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G24" t="n">
+        <v>5.821103448275863</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>void ck::kernel_moe_mxgemm_2lds&lt;ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleExpertWeightShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 256, 64, 128, 128, 16, 16, 16, 16, 4, 2, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 8, 1, 32&gt;, ck::Sequence&lt;2, 1, 2&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)2, 0, false, false, true, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;, true, (ck::InMemoryDataOperationEnum)1, 2, (ck::TailNumber)1&gt;(ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleExpertWeightShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 256, 64, 128, 128, 16, 16, 16, 16, 4, 2, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 8, 1, 32&gt;, ck::Sequence&lt;2, 1, 2&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)2, 0, false, false, true, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;::Argument)</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>63.679</v>
+      </c>
+      <c r="D25" t="n">
+        <v>16.1</v>
+      </c>
+      <c r="G25" t="n">
+        <v>57.9661724137931</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="n">
-        <v>86.27600000000001</v>
-      </c>
-      <c r="D6" t="n">
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="n">
+        <v>395.459</v>
+      </c>
+      <c r="D26" t="n">
         <v>100</v>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="n">
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="n">
         <v>100</v>
       </c>
-      <c r="G6" t="n">
-        <v>61.21382926829268</v>
-      </c>
-      <c r="H6" t="inlineStr"/>
+      <c r="G26" t="n">
+        <v>399.4528103448276</v>
+      </c>
+      <c r="H26" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="28">
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="E19:E25"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="E10:E11"/>
     <mergeCell ref="F2:F3"/>
+    <mergeCell ref="H19:H25"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="H7:H8"/>
     <mergeCell ref="E2:E3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="F19:F25"/>
+    <mergeCell ref="A19:A25"/>
+    <mergeCell ref="H12:H13"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="H10:H11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -604,7 +1074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -637,77 +1107,381 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>void aiter::reduce_scatter_cross_device_store&lt;std::bfloat16_t, 4&gt;(aiter::RankData*, aiter::RankSignals, aiter::Signal*, int, int)</t>
+          <t>void ck::kernel_moe_mxgemm_2lds&lt;ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 256, 64, 128, 128, 16, 16, 16, 16, 4, 2, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 32, 1, 8&gt;, ck::Sequence&lt;8, 1, 8&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)2, 1, false, true, false, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;, true, (ck::InMemoryDataOperationEnum)0, 2, (ck::TailNumber)1&gt;(ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 256, 64, 128, 128, 16, 16, 16, 16, 4, 2, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 32, 1, 8&gt;, ck::Sequence&lt;8, 1, 8&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)2, 1, false, true, false, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;::Argument)</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>56.639</v>
+        <v>123.76</v>
       </c>
       <c r="D2" t="n">
-        <v>56.639</v>
+        <v>123.76</v>
       </c>
       <c r="E2" t="n">
-        <v>65.59999999999999</v>
+        <v>31.3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>aiter::bf16gemm_fp32bf16_tn_64x64_splitk_clean</t>
+          <t>void ck::kernel_moe_mxgemm_2lds&lt;ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleExpertWeightShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 256, 64, 128, 128, 16, 16, 16, 16, 4, 2, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 8, 1, 32&gt;, ck::Sequence&lt;2, 1, 2&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)2, 0, false, false, true, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;, true, (ck::InMemoryDataOperationEnum)1, 2, (ck::TailNumber)1&gt;(ck::GridwiseMoeGemmMX_BPreshuffle&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::Tuple&lt;ck::tensor_layout::gemm::RowMajor, ck::tensor_layout::gemm::ColumnMajor, ck::tensor_layout::gemm::RowMajor&gt;, ck::tensor_layout::gemm::RowMajor, ck::f4x2_pk_t, ck::e8m0_bexp_t, ck::f4x2_pk_t, ck::e8m0_bexp_t, float, float, ck::Tuple&lt;float, float, float&gt;, unsigned short, ck::tensor_operation::element_wise::PassThrough, ck::tensor_operation::element_wise::PassThrough, MulABScaleExpertWeightShuffled, (ck::tensor_operation::device::GemmSpecialization)0, 32, 256, 64, 128, 128, 16, 16, 16, 16, 4, 2, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, ck::Sequence&lt;8, 32, 1&gt;, ck::Sequence&lt;1, 0, 2&gt;, ck::Sequence&lt;1, 0, 2&gt;, 2, 16, 16, false, 1, 2, 2, ck::Sequence&lt;1, 8, 1, 32&gt;, ck::Sequence&lt;2, 1, 2&gt;, (ck::BlockGemmPipelineScheduler)0, (ck::BlockGemmPipelineVersion)2, 0, false, false, true, int, ck::f4x2_pk_t, ck::f4x2_pk_t&gt;::Argument)</t>
         </is>
       </c>
       <c r="B3" t="n">
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>18.279</v>
+        <v>63.679</v>
       </c>
       <c r="D3" t="n">
-        <v>18.279</v>
+        <v>63.679</v>
       </c>
       <c r="E3" t="n">
-        <v>21.2</v>
+        <v>16.1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>void aiter::local_device_load_rmsnorm&lt;std::bfloat16_t, 512, 2&gt;(aiter::RankSignals, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, float, int, int, int)</t>
+          <t>void aiter::reduce_scatter_cross_device_store&lt;std::bfloat16_t, 4&gt;(aiter::RankData*, aiter::RankSignals, aiter::Signal*, int, int)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C4" t="n">
-        <v>5.719</v>
+        <v>35.718</v>
       </c>
       <c r="D4" t="n">
-        <v>5.719</v>
+        <v>17.859</v>
       </c>
       <c r="E4" t="n">
-        <v>6.6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>aiter::mla_a8w8_qh16_qseqlen1_gqaratio16_ps</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>25.319</v>
+      </c>
+      <c r="D5" t="n">
+        <v>25.319</v>
+      </c>
+      <c r="E5" t="n">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>aiter::bf16gemm_fp32bf16_tn_64x64_splitk_clean</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>25.16</v>
+      </c>
+      <c r="D6" t="n">
+        <v>12.58</v>
+      </c>
+      <c r="E6" t="n">
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Cijk_Alik_Bljk_BBS_BH_Bias_HA_S_SAV_UserArgs_MT64x64x128_MI16x16x1_SN_LDSB1_AFC1_AFEM1_AFEM1_ASEM1_CLR1_CADS0_DTLA0_DTLB0_DTVA0_DTVB0_EPS0_FDSI0_GRPM1_GRVWA8_GRVWB8_GSU0_GSUAMB_GLS0_ISA950_IU1_K1_LBSPPA512_LBSPPB512_LBSPPM0_LPA16_LPB16_LPM0_LRVW8_LWPMn1_MIAV0_MIWT2_2_MO40_NTn1_NTA0_NTB0_NTC0_NTD0_NTM0_NEPBS0_NLCA1_NLCB1_ONLL1_PGR2_PLR1_PKA1_SIA3_SS1_SPO0_SRVW0_SSO0_SVW2_SK3_SKXCCM8_TLDS1_ULSGRO0_USL1_UIOFGRO0_USFGRO0_VSn1_VWA2_VWB2_WSGRA0_WSGRB0_WS64_WG32_8_1</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>20.279</v>
+      </c>
+      <c r="D7" t="n">
+        <v>20.279</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>_fused_dynamic_mxfp4_quant_moe_sort_kernel</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>15.598</v>
+      </c>
+      <c r="D8" t="n">
+        <v>7.799</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cijk_Alik_Bljk_BBS_BH_Bias_HA_S_SAV_UserArgs_MT64x32x128_MI16x16x1_SN_LDSB1_AFC1_AFEM1_AFEM1_ASEM1_CLR1_CADS0_DTLA0_DTLB0_DTVA0_DTVB0_EPS0_FDSI0_GRPM1_GRVWA8_GRVWB8_GSU0_GSUAMB_GLS0_ISA950_IU1_K1_LBSPPA512_LBSPPB256_LBSPPM0_LPA16_LPB16_LPM0_LRVW8_LWPMn1_MIAV0_MIWT2_1_MO40_NTn1_NTA0_NTB0_NTC0_NTD0_NTM0_NEPBS0_NLCA1_NLCB1_ONLL1_PGR2_PLR1_PKA1_SIA3_SS1_SPO0_SRVW0_SSO0_SVW2_SK3_SKXCCM8_TLDS1_ULSGRO0_USL1_UIOFGRO0_USFGRO0_VSn1_VWA2_VWB1_WSGRA0_WSGRB0_WS64_WG32_8_1</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="n">
+        <v>10.879</v>
+      </c>
+      <c r="D9" t="n">
+        <v>10.879</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>void aiter::local_device_load_rmsnorm&lt;std::bfloat16_t, 512, 2&gt;(aiter::RankSignals, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, float, int, int, int)</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10.798</v>
+      </c>
+      <c r="D10" t="n">
+        <v>5.399</v>
+      </c>
+      <c r="E10" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>void kn_mla_reduce_v1_ps&lt;MlaReduceKernelV1Traits&lt;512, 16, 1&gt;, float, std::bfloat16_t&gt;(MlaReduceKernelV1Params)</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" t="n">
+        <v>6.599</v>
+      </c>
+      <c r="D11" t="n">
+        <v>6.599</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>void ck_tile::kentry&lt;2, ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;, ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;::Kargs&gt;(ck_tile::MoeSortingMultiPhaseKernel_P0_v2&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;::Kargs)</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" t="n">
+        <v>6.519</v>
+      </c>
+      <c r="D12" t="n">
+        <v>6.519</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>void ck_tile::kentry&lt;2, ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;, ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;::Kargs&gt;(ck_tile::MoeSortingMultiPhaseKernel_P23&lt;ck_tile::MoeSortingProblemMp&lt;int, float, int, 1, true, false, true&gt; &gt;::Kargs)</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1</v>
+      </c>
+      <c r="C13" t="n">
+        <v>6.519</v>
+      </c>
+      <c r="D13" t="n">
+        <v>6.519</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>triton_poi_fused_as_strided_clone_copy__0</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>6.479</v>
+      </c>
+      <c r="D14" t="n">
+        <v>6.479</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>void aiter::add_rmsnorm_quant_kernel&lt;std::bfloat16_t, std::bfloat16_t, 64, 8, false, false, true, 1&gt;(std::bfloat16_t*, std::bfloat16_t*, float*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, double, int, int, int, int, int, int, int, bool)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="D15" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>_batched_gemm_a8w8_a_per_token_group_prequant_w_per_batched_tensor_quant_kernel_HAS_BIAS_0_BLOCK_SIZE_M_32_BLOCK_SIZE_N_128_BLOCK_SIZE_K_128_GROUP_SIZE_M_1_EVEN_K_1_EVEN_MN_1_cache_modifier_CG</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="D16" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>triton_poi_fused_as_strided_clone_1</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="D17" t="n">
+        <v>5.519</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>void aiter::add_rmsnorm_quant_kernel&lt;std::bfloat16_t, std::bfloat16_t, 256, 8, false, false, true, 1&gt;(std::bfloat16_t*, std::bfloat16_t*, float*, std::bfloat16_t*, std::bfloat16_t*, std::bfloat16_t*, double, int, int, int, int, int, int, int, bool)</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>5.639</v>
-      </c>
-      <c r="D5" t="n">
-        <v>5.639</v>
-      </c>
-      <c r="E5" t="n">
-        <v>6.5</v>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>5.479</v>
+      </c>
+      <c r="D18" t="n">
+        <v>5.479</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>_batched_gemm_a8w8_a_per_token_group_prequant_w_per_batched_tensor_quant_kernel_HAS_BIAS_0_BLOCK_SIZE_M_32_BLOCK_SIZE_N_64_BLOCK_SIZE_K_128_GROUP_SIZE_M_1_EVEN_K_1_EVEN_MN_1_cache_modifier_CG</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>1</v>
+      </c>
+      <c r="C19" t="n">
+        <v>5.439</v>
+      </c>
+      <c r="D19" t="n">
+        <v>5.439</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>void aiter::fuse_qk_rope_concat_and_cache_mla_per_head_kernel&lt;std::bfloat16_t, _BitInt(8), _BitInt(8), (vllm::Fp8KVCacheDataType)1, (vllm::Fp8KVCacheDataType)1, 8&gt;(std::bfloat16_t const*, std::bfloat16_t const*, std::bfloat16_t const*, std::bfloat16_t const*, _BitInt(8)*, _BitInt(8)*, long const*, long const*, std::bfloat16_t const*, std::bfloat16_t const*, int, int, int, int, int, int, int, int, int, int, int, int, int, int, float const*, float const*, bool, bool)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>5.359</v>
+      </c>
+      <c r="D20" t="n">
+        <v>5.359</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>void aiter::grouped_topk_opt_sort_kernel&lt;c10::BFloat16, float __vector(4), 8, true, true, false&gt;(c10::BFloat16*, c10::BFloat16 const*, float*, int*, unsigned long, int, int, int, int, float)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>1</v>
+      </c>
+      <c r="C21" t="n">
+        <v>5.319</v>
+      </c>
+      <c r="D21" t="n">
+        <v>5.319</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>